<commit_message>
changed automatic case pack recommendation price logic
</commit_message>
<xml_diff>
--- a/config/items.xlsx
+++ b/config/items.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan\Desktop\barcodeUtils\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7664546F-05CB-46DE-9D7B-6CBDE90AA928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B8EFCF-E9A2-4676-92CE-4BCF6F1ADF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="28800" windowHeight="15435" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15435" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -105,10 +105,10 @@
     <t>SI</t>
   </si>
   <si>
-    <t>N305</t>
-  </si>
-  <si>
-    <t>N305-EXPRIMIDOR DE NARANJA MANUAL</t>
+    <t>S164-TETERA -HERVIDORA PIEDRA VOLCANICA</t>
+  </si>
+  <si>
+    <t>S164</t>
   </si>
 </sst>
 </file>
@@ -544,10 +544,10 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
         <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
       </c>
       <c r="E2" t="s">
         <v>20</v>
@@ -556,7 +556,7 @@
         <v>21</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H2">
         <v>10</v>
@@ -574,10 +574,10 @@
         <v>0</v>
       </c>
       <c r="P2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T2" t="s">
         <v>24</v>
-      </c>
-      <c r="T2" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Html References fixed saveSheet visibility
</commit_message>
<xml_diff>
--- a/config/items.xlsx
+++ b/config/items.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan\Desktop\barcodeUtils\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan\Desktop\barcodeutils\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B8EFCF-E9A2-4676-92CE-4BCF6F1ADF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8956D135-B0A6-46DD-9D68-2888FEDBDE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15435" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -105,10 +105,10 @@
     <t>SI</t>
   </si>
   <si>
-    <t>S164-TETERA -HERVIDORA PIEDRA VOLCANICA</t>
-  </si>
-  <si>
     <t>S164</t>
+  </si>
+  <si>
+    <t>S164-Zapatera</t>
   </si>
 </sst>
 </file>
@@ -544,10 +544,10 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
       </c>
       <c r="E2" t="s">
         <v>20</v>
@@ -556,7 +556,7 @@
         <v>21</v>
       </c>
       <c r="G2">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H2">
         <v>10</v>
@@ -574,10 +574,10 @@
         <v>0</v>
       </c>
       <c r="P2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T2" t="s">
         <v>23</v>
-      </c>
-      <c r="T2" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>